<commit_message>
VOYAP yangın rev: Aselsan 02-Yangın lejant sembolleri, çap tablosu (DN25-DN150, ana kolon SP-1 DN150), tüm başlıklar çizili, mimari planlar dahil TAM pafta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/voyap_yangin/VOYAP_YANGIN_HESAP.xlsx
+++ b/proje/voyap_yangin/VOYAP_YANGIN_HESAP.xlsx
@@ -1155,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1281,10 +1281,10 @@
         <v>1044</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>1.92</v>
+        <v>1.9</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>61</v>
@@ -1410,7 +1410,7 @@
         <v>1.3</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>2.92</v>
+        <v>2.91</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>67</v>
@@ -1463,17 +1463,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>4"</t>
+          <t>DN150</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>105.3</v>
+        <v>155.4</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>32.27</v>
+        <v>3.34</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>1044</v>
@@ -1490,17 +1490,17 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>3"</t>
+          <t>DN100</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>80.90000000000001</v>
+        <v>105.3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>12</v>
+        <v>28.93</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>1044</v>
@@ -1517,20 +1517,20 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2 1/2"</t>
+          <t>DN80</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>68.90000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>927.9</v>
+        <v>1044</v>
       </c>
       <c r="F13" s="8">
         <f>6.05E5*E13^1.85/(120^1.85*C13^4.87)*D13*1.2</f>
@@ -1544,7 +1544,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2 1/2"</t>
+          <t>DN65</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -1557,7 +1557,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>692.6</v>
+        <v>927.9</v>
       </c>
       <c r="F14" s="8">
         <f>6.05E5*E14^1.85/(120^1.85*C14^4.87)*D14*1.2</f>
@@ -1571,20 +1571,20 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN65</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>53.1</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>407.7</v>
+        <v>692.6</v>
       </c>
       <c r="F15" s="8">
         <f>6.05E5*E15^1.85/(120^1.85*C15^4.87)*D15*1.2</f>
@@ -1598,7 +1598,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -1608,10 +1608,10 @@
         <v>53.1</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.72</v>
+        <v>3</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>351.6</v>
+        <v>407.7</v>
       </c>
       <c r="F16" s="8">
         <f>6.05E5*E16^1.85/(120^1.85*C16^4.87)*D16*1.2</f>
@@ -1625,7 +1625,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -1635,10 +1635,10 @@
         <v>53.1</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.62</v>
+        <v>0.72</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>294</v>
+        <v>351.6</v>
       </c>
       <c r="F17" s="8">
         <f>6.05E5*E17^1.85/(120^1.85*C17^4.87)*D17*1.2</f>
@@ -1652,20 +1652,20 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>1 1/2"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>41.9</v>
+        <v>53.1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>3</v>
+        <v>0.62</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>192.8</v>
+        <v>294</v>
       </c>
       <c r="F18" s="8">
         <f>6.05E5*E18^1.85/(120^1.85*C18^4.87)*D18*1.2</f>
@@ -1679,20 +1679,20 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN40</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>27.3</v>
+        <v>41.9</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.61</v>
+        <v>3</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>97.3</v>
+        <v>192.8</v>
       </c>
       <c r="F19" s="8">
         <f>6.05E5*E19^1.85/(120^1.85*C19^4.87)*D19*1.2</f>
@@ -1706,7 +1706,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN25</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
@@ -1716,10 +1716,10 @@
         <v>27.3</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>3.02</v>
+        <v>0.61</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>47.3</v>
+        <v>97.3</v>
       </c>
       <c r="F20" s="8">
         <f>6.05E5*E20^1.85/(120^1.85*C20^4.87)*D20*1.2</f>
@@ -1731,101 +1731,101 @@
       </c>
     </row>
     <row r="21">
-      <c r="E21" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>DN25</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="F21" s="8">
+        <f>6.05E5*E21^1.85/(120^1.85*C21^4.87)*D21*1.2</f>
+        <v/>
+      </c>
+      <c r="G21" s="8">
+        <f>E21/60000/(PI()*(C21/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Toplam</t>
         </is>
       </c>
-      <c r="F21" s="9">
-        <f>SUM(F11:F20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="F22" s="9">
+        <f>SUM(F11:F21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>ZEMİN KAT - kat girişinden en uzak başlığa boru yolu</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Çap</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>DN</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>İç çap mm</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>L m</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>Q l/dk</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Δp bar</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>v m/s</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>4"</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>105.3</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>30.71</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>867.3</v>
-      </c>
-      <c r="F25" s="8">
-        <f>6.05E5*E25^1.85/(120^1.85*C25^4.87)*D25*1.2</f>
-        <v/>
-      </c>
-      <c r="G25" s="8">
-        <f>E25/60000/(PI()*(C25/1000)^2/4)</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>3"</t>
+          <t>DN100</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>80.90000000000001</v>
+        <v>105.3</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>9</v>
+        <v>30.71</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>867.3</v>
@@ -1842,20 +1842,20 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2 1/2"</t>
+          <t>DN80</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>68.90000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>717.5</v>
+        <v>867.3</v>
       </c>
       <c r="F27" s="8">
         <f>6.05E5*E27^1.85/(120^1.85*C27^4.87)*D27*1.2</f>
@@ -1869,20 +1869,20 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN65</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>53.1</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>493.7</v>
+        <v>717.5</v>
       </c>
       <c r="F28" s="8">
         <f>6.05E5*E28^1.85/(120^1.85*C28^4.87)*D28*1.2</f>
@@ -1896,7 +1896,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -1906,10 +1906,10 @@
         <v>53.1</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.12</v>
+        <v>3</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>419.4</v>
+        <v>493.7</v>
       </c>
       <c r="F29" s="8">
         <f>6.05E5*E29^1.85/(120^1.85*C29^4.87)*D29*1.2</f>
@@ -1923,20 +1923,20 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>1 1/2"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>41.9</v>
+        <v>53.1</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>2.4</v>
+        <v>0.12</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>267.3</v>
+        <v>419.4</v>
       </c>
       <c r="F30" s="8">
         <f>6.05E5*E30^1.85/(120^1.85*C30^4.87)*D30*1.2</f>
@@ -1950,20 +1950,20 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN40</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>27.3</v>
+        <v>41.9</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>2.98</v>
+        <v>2.4</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>123.2</v>
+        <v>267.3</v>
       </c>
       <c r="F31" s="8">
         <f>6.05E5*E31^1.85/(120^1.85*C31^4.87)*D31*1.2</f>
@@ -1977,7 +1977,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN25</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
@@ -1987,10 +1987,10 @@
         <v>27.3</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>3.02</v>
+        <v>2.98</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>60</v>
+        <v>123.2</v>
       </c>
       <c r="F32" s="8">
         <f>6.05E5*E32^1.85/(120^1.85*C32^4.87)*D32*1.2</f>
@@ -2002,101 +2002,101 @@
       </c>
     </row>
     <row r="33">
-      <c r="E33" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DN25</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F33" s="8">
+        <f>6.05E5*E33^1.85/(120^1.85*C33^4.87)*D33*1.2</f>
+        <v/>
+      </c>
+      <c r="G33" s="8">
+        <f>E33/60000/(PI()*(C33/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Toplam</t>
         </is>
       </c>
-      <c r="F33" s="9">
-        <f>SUM(F25:F32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="F34" s="9">
+        <f>SUM(F26:F33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>1. KAT - kat girişinden en uzak başlığa boru yolu</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>Çap</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>DN</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>İç çap mm</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>L m</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>Q l/dk</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Δp bar</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>v m/s</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>4"</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>105.3</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>30.98</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>424.3</v>
-      </c>
-      <c r="F37" s="8">
-        <f>6.05E5*E37^1.85/(120^1.85*C37^4.87)*D37*1.2</f>
-        <v/>
-      </c>
-      <c r="G37" s="8">
-        <f>E37/60000/(PI()*(C37/1000)^2/4)</f>
-        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>3"</t>
+          <t>DN150</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>80.90000000000001</v>
+        <v>155.4</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>11.26</v>
+        <v>1.52</v>
       </c>
       <c r="E38" s="4" t="n">
         <v>424.3</v>
@@ -2113,20 +2113,20 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>2 1/2"</t>
+          <t>DN100</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>68.90000000000001</v>
+        <v>105.3</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>7.13</v>
+        <v>29.46</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>345.6</v>
+        <v>424.3</v>
       </c>
       <c r="F39" s="8">
         <f>6.05E5*E39^1.85/(120^1.85*C39^4.87)*D39*1.2</f>
@@ -2140,20 +2140,20 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN80</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>53.1</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>8.44</v>
+        <v>11.26</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>345.6</v>
+        <v>424.3</v>
       </c>
       <c r="F40" s="8">
         <f>6.05E5*E40^1.85/(120^1.85*C40^4.87)*D40*1.2</f>
@@ -2167,20 +2167,20 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>1 1/2"</t>
+          <t>DN65</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>41.9</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>3.28</v>
+        <v>7.13</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>269.2</v>
+        <v>345.6</v>
       </c>
       <c r="F41" s="8">
         <f>6.05E5*E41^1.85/(120^1.85*C41^4.87)*D41*1.2</f>
@@ -2194,20 +2194,20 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C42" s="4" t="n">
-        <v>27.3</v>
+        <v>53.1</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>3.27</v>
+        <v>8.44</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>123.2</v>
+        <v>345.6</v>
       </c>
       <c r="F42" s="8">
         <f>6.05E5*E42^1.85/(120^1.85*C42^4.87)*D42*1.2</f>
@@ -2221,20 +2221,20 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN40</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>27.3</v>
+        <v>41.9</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>3.02</v>
+        <v>3.28</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>60</v>
+        <v>269.2</v>
       </c>
       <c r="F43" s="8">
         <f>6.05E5*E43^1.85/(120^1.85*C43^4.87)*D43*1.2</f>
@@ -2246,131 +2246,131 @@
       </c>
     </row>
     <row r="44">
-      <c r="E44" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DN25</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>123.2</v>
+      </c>
+      <c r="F44" s="8">
+        <f>6.05E5*E44^1.85/(120^1.85*C44^4.87)*D44*1.2</f>
+        <v/>
+      </c>
+      <c r="G44" s="8">
+        <f>E44/60000/(PI()*(C44/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>DN25</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F45" s="8">
+        <f>6.05E5*E45^1.85/(120^1.85*C45^4.87)*D45*1.2</f>
+        <v/>
+      </c>
+      <c r="G45" s="8">
+        <f>E45/60000/(PI()*(C45/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="E46" t="inlineStr">
         <is>
           <t>Toplam</t>
         </is>
       </c>
-      <c r="F44" s="9">
-        <f>SUM(F37:F43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="F46" s="9">
+        <f>SUM(F38:F45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>2. KAT - kat girişinden en uzak başlığa boru yolu</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>Çap</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>DN</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>İç çap mm</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>L m</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>Q l/dk</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>Δp bar</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G49" s="7" t="inlineStr">
         <is>
           <t>v m/s</t>
         </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>4"</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C48" s="4" t="n">
-        <v>105.3</v>
-      </c>
-      <c r="D48" s="4" t="n">
-        <v>30.98</v>
-      </c>
-      <c r="E48" s="4" t="n">
-        <v>424.3</v>
-      </c>
-      <c r="F48" s="8">
-        <f>6.05E5*E48^1.85/(120^1.85*C48^4.87)*D48*1.2</f>
-        <v/>
-      </c>
-      <c r="G48" s="8">
-        <f>E48/60000/(PI()*(C48/1000)^2/4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>3"</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="C49" s="4" t="n">
-        <v>80.90000000000001</v>
-      </c>
-      <c r="D49" s="4" t="n">
-        <v>11.26</v>
-      </c>
-      <c r="E49" s="4" t="n">
-        <v>424.3</v>
-      </c>
-      <c r="F49" s="8">
-        <f>6.05E5*E49^1.85/(120^1.85*C49^4.87)*D49*1.2</f>
-        <v/>
-      </c>
-      <c r="G49" s="8">
-        <f>E49/60000/(PI()*(C49/1000)^2/4)</f>
-        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2 1/2"</t>
+          <t>DN150</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>68.90000000000001</v>
+        <v>155.4</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>7.13</v>
+        <v>1.52</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>345.6</v>
+        <v>424.3</v>
       </c>
       <c r="F50" s="8">
         <f>6.05E5*E50^1.85/(120^1.85*C50^4.87)*D50*1.2</f>
@@ -2384,20 +2384,20 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN100</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>53.1</v>
+        <v>105.3</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>8.44</v>
+        <v>29.46</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>345.6</v>
+        <v>424.3</v>
       </c>
       <c r="F51" s="8">
         <f>6.05E5*E51^1.85/(120^1.85*C51^4.87)*D51*1.2</f>
@@ -2411,20 +2411,20 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>1 1/2"</t>
+          <t>DN80</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>41.9</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>3.28</v>
+        <v>11.26</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>269.2</v>
+        <v>424.3</v>
       </c>
       <c r="F52" s="8">
         <f>6.05E5*E52^1.85/(120^1.85*C52^4.87)*D52*1.2</f>
@@ -2438,20 +2438,20 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN65</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="C53" s="4" t="n">
-        <v>27.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D53" s="4" t="n">
-        <v>3.27</v>
+        <v>7.13</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>123.2</v>
+        <v>345.6</v>
       </c>
       <c r="F53" s="8">
         <f>6.05E5*E53^1.85/(120^1.85*C53^4.87)*D53*1.2</f>
@@ -2465,20 +2465,20 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C54" s="4" t="n">
-        <v>27.3</v>
+        <v>53.1</v>
       </c>
       <c r="D54" s="4" t="n">
-        <v>3.02</v>
+        <v>8.44</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>60</v>
+        <v>345.6</v>
       </c>
       <c r="F54" s="8">
         <f>6.05E5*E54^1.85/(120^1.85*C54^4.87)*D54*1.2</f>
@@ -2490,13 +2490,94 @@
       </c>
     </row>
     <row r="55">
-      <c r="E55" t="inlineStr">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>DN40</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>269.2</v>
+      </c>
+      <c r="F55" s="8">
+        <f>6.05E5*E55^1.85/(120^1.85*C55^4.87)*D55*1.2</f>
+        <v/>
+      </c>
+      <c r="G55" s="8">
+        <f>E55/60000/(PI()*(C55/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>DN25</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>123.2</v>
+      </c>
+      <c r="F56" s="8">
+        <f>6.05E5*E56^1.85/(120^1.85*C56^4.87)*D56*1.2</f>
+        <v/>
+      </c>
+      <c r="G56" s="8">
+        <f>E56/60000/(PI()*(C56/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>DN25</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C57" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F57" s="8">
+        <f>6.05E5*E57^1.85/(120^1.85*C57^4.87)*D57*1.2</f>
+        <v/>
+      </c>
+      <c r="G57" s="8">
+        <f>E57/60000/(PI()*(C57/1000)^2/4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Toplam</t>
         </is>
       </c>
-      <c r="F55" s="9">
-        <f>SUM(F48:F54)</f>
+      <c r="F58" s="9">
+        <f>SUM(F50:F57)</f>
         <v/>
       </c>
     </row>
@@ -2511,7 +2592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2571,7 +2652,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>DN25</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -2594,7 +2675,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1 1/4"</t>
+          <t>DN32</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -2617,7 +2698,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>1 1/2"</t>
+          <t>DN40</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -2640,7 +2721,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2"</t>
+          <t>DN50</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -2663,7 +2744,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2 1/2"</t>
+          <t>DN65</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -2686,7 +2767,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3"</t>
+          <t>DN80</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -2709,66 +2790,74 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>4"</t>
+          <t>DN100</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>32.3</v>
+        <v>28.9</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>30.7</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>31</v>
+        <v>29.5</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>31</v>
+        <v>29.5</v>
       </c>
       <c r="F10" s="10">
         <f>SUM(B10:E10)</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DN150</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F11" s="10">
+        <f>SUM(B11:E11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>MALZEME</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>MİKTAR</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>BİRİM</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Sprinkler upright K80 68°C</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>214</v>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>adet</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Sprinkler pendant K80 68°C</t>
+          <t>Sprinkler upright K80 68°C</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>244</v>
+        <v>214</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
@@ -2779,11 +2868,11 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Ara seviye sprinkler (lift)</t>
+          <t>Sprinkler pendant K80 68°C</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>22</v>
+        <v>244</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
@@ -2794,11 +2883,11 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Yangın dolabı TS EN 671-1</t>
+          <t>Ara seviye sprinkler (lift)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
@@ -2809,11 +2898,11 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Islak alarm vanası DN100</t>
+          <t>Yangın dolabı TS EN 671-1</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
@@ -2824,37 +2913,37 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Kat kontrol istasyonu DN100</t>
+          <t>Islak alarm vanası DN100</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>takım</t>
+          <t>adet</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>İtfaiye bağlantısı 2x2½"</t>
+          <t>Kat kontrol istasyonu DN100</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>adet</t>
+          <t>takım</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Yangın pompa grubu (E+D+J)</t>
+          <t>İtfaiye bağlantısı 2x2½"</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
@@ -2862,14 +2951,14 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>takım</t>
+          <t>adet</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Yangın suyu deposu 80 m³</t>
+          <t>Yangın pompa grubu (E+D+J)</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
@@ -2877,20 +2966,35 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>adet</t>
+          <t>takım</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Yedek sprinkler dolabı (6 adet başlık + anahtar)</t>
+          <t>Yangın suyu deposu 80 m³</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>adet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Yedek sprinkler dolabı (6 adet başlık + anahtar)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>adet</t>
         </is>

</xml_diff>